<commit_message>
Update Test Case Postman
</commit_message>
<xml_diff>
--- a/Calculator/CalculatorTester/Data/DataSet.xlsx
+++ b/Calculator/CalculatorTester/Data/DataSet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiemThuPM\DemoTesterVerC-\Calculator\CalculatorTester\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08580635-62ED-4ED7-86C1-CB0E485DFE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C9FE5C-DB2E-4356-827D-D06DF3EDDC5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0DEF87D9-2C7E-4447-B58F-0DEE76119D00}"/>
+    <workbookView xWindow="9408" yWindow="2544" windowWidth="12900" windowHeight="8880" xr2:uid="{0DEF87D9-2C7E-4447-B58F-0DEE76119D00}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -104,6 +104,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -459,58 +462,58 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="4">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="4">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="4">
         <v>3</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="4">
         <v>-1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="A4" s="4">
         <v>4</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="4">
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="4">
         <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+      <c r="A5" s="4">
         <v>5</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="4">
         <v>5</v>
       </c>
       <c r="C5" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
     </row>

</xml_diff>